<commit_message>
Show sibling table rows so ambiguity can be judged without the source PDFs
Judging whether the gold answer is the only defensible one mostly comes down to
whether a competing line item sits in the same table -- 归属于上市公司股东的净资产
next to 所有者权益合计, 营业收入 next to 营业总收入. That is answerable from the
corpus, so the sheet now carries the neighbouring rows and their values, ranked
by character overlap with the queried indicator. 85 of the 100 random items and
66 of the 80 hard ones become decidable without opening a PDF, which matters
because the 103 source reports are 859 MB and are not in the repository.

agreement.py now locates the judgment columns by header text. Adding a column
shifted them from H/I to I/J, and a hard-coded letter would have read empty
cells and reported perfect agreement instead of failing. It also tolerates the
first-round sheet, whose format predates this column set.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/抽检表_标注者A.xlsx
+++ b/抽检表_标注者A.xlsx
@@ -479,19 +479,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,7 +508,8 @@
           <t>填写说明：只需填黄色三列，用下拉选择 ✓ / ✗ / 存疑，有疑问时在备注列写一句原因。第4行为示例行（不计入统计）。请独立判定——不要参考另一位标注者的结果，也不要互相商量，否则一致性系数失去意义。
 【答案正确?】标准答案与原文是否相符（数值、行标签、年份、量纲）。相符✓，不符✗。
 【唯一合理答案?】在问题的字面表述下，标准答案是否是唯一站得住的答案。是✓；若一个称职的分析师可能给出另一个同样站得住的答案，判✗并在备注写出那个答案。常见歧义来源：①指标口径（归母净资产／所有者权益合计、营业收入／营业总收入）；②合并报表与母公司报表；③上年数是追溯调整后还是原披露数；④同一年数字在本年报与次年年报的上年同期栏都出现，取哪一处。
-注意这两列相互独立：答案可以完全正确，但问题本身有歧义（判 ✓ / ✗）。证据原文列是自动匹配的 gold 三元组；表名若读不出计量单位，请对照原PDF确认量纲。
+注意这两列相互独立：答案可以完全正确，但问题本身有歧义。
+【同表相近行】列出了同一张表里口径相近的其他科目及其数值——判歧义时先看这一列，多数情况无需打开源PDF。仅当表名读不出计量单位、或需确认上年数是否追溯调整时，才需对照原PDF。
 本页刻意挑选了核验成本高或存在分歧风险的条目（证据跨表跨页、单位由表名回挂、比率类指标等）。顺序已打散，判定时无需考虑它为何入选。</t>
         </is>
       </c>
@@ -545,20 +547,25 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>同表相近行（判歧义用）</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>来源（文件@页）</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>答案正确?</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>唯一合理答案?</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -597,22 +604,28 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
+          <t>营业总收入 = 164,699百万元
+利息净收入 = 116,061百万元</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
           <t>000001_平安银行_2023年年度报告.pdf @15</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>数值与原文一致；「营业收入」在该表中口径唯一</t>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>数值与原文一致；该表虽有「营业总收入」，但本行两者同值，不构成歧义</t>
         </is>
       </c>
     </row>
@@ -648,12 +661,18 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 62,791,872,697.72元
+归属于上市公司股 东的净资产 = 197,506,672,396.00元</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -689,12 +708,19 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 21.34%
+归属于上市公司股东的净资产（元） = 69,327,010,925.99
+归属于上市公司股东的净资产 = 53,179,935,140.80元</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
           <t>002475_立讯精密_2024年年度报告.pdf @8; 600887_伊利股份_内蒙古伊利实业集团股份有限公司2024年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -728,12 +754,17 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的净资产 = 197,506,672,396.00元</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -769,12 +800,17 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
           <t>600276_恒瑞医药_恒瑞医药2023年年度报告.pdf @6; 600276_恒瑞医药_恒瑞医药2024年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -810,12 +846,22 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的每股净资产 = 21.00
+全面摊薄净资产收 益率 = 9.32%
+加权平均净资产收 益率 = 9.48%
+加权平均净资产收益率 = 25.28%
+归属于上市公司股 东的净利润 = 22,617,778,516.45元
+归属于上市公司股 东的扣除非经常性 损益的净利润 = 19,762,103,017.38元</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
           <t>000002_万科A_2022年年度报告.pdf @12; 000858_五 粮 液_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -849,12 +895,17 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2023年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -890,12 +941,17 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 4,141,262,764.05元</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
           <t>002594_比亚迪_2022年年度报告.pdf @8; 600276_恒瑞医药_恒瑞医药2023年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -931,12 +987,22 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每 股收益（元／股） = 59.51
+扣除非经常性损益后的基本每股 收益（元／股） = 49.99
+稀释每股收益（元／股） = 59.49
+加权平均净资产收益率（%） = 34.19
+扣除非经常性损益后的加权平 均净资产收益率（%） = 34.20
+扣除非经常性损益后的加权平均 净资产收益率（%） = 30.29</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2022年年度报告.pdf @5; 600519_贵州茅台_贵州茅台2023年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -972,12 +1038,20 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 9,747,587,804.59元
+归属于上市公司股东的扣 除非经常性损益的净利润 = 8,260,289,685.19元
+归属于上市公司股 东的净资产 = 55,122,453,910.73元
+归属于上市公司股东的净 资产 = 46,589,953,393.31元</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2022年年度报告.pdf @7; 603259_药明康德_2023年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr"/>
       <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1011,12 +1085,20 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每股收益（元／股） = 1.34
+稀释每股收益（元／股） = 1.48
+加权平均净资产收益率（%） = 19.23
+扣除非经常性损益后的加权平均净资产收益率（%） = 17.39</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
           <t>600887_伊利股份_内蒙古伊利实业集团股份有限公司2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr"/>
       <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -1050,12 +1132,20 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
+          <t>稀释每股收益 = (4.17)
+扣除非经常性损益后归属于上 市公司股东的净利润 = (45,393,719,289.83)元
+净资产收益率（全面摊薄） = -24.41%
+净资产收益率（加权平均） = -21.82%</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
           <t>000002_万科A_2024年年度报告.pdf @11</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr"/>
       <c r="I15" s="6" t="inlineStr"/>
       <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1089,12 +1179,17 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
           <t>601088_中国神华_中国神华2025年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr"/>
       <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -1128,12 +1223,17 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东 的扣除非经常性损益 的净利润（元） = 8,068,550,808.00</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
           <t>300760_迈瑞医疗_2025年年度报告.pdf @20</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr"/>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -1167,12 +1267,20 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净 利润 = 8,813,713,033.51元
+归属于上市公司股东的扣 除非经常性损益的净利润 = 8,260,289,685.19元
+经营活动产生的现金流量 净额 = 10,616,029,916.68元
+总资产 = 64,690,326,746.96元</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
@@ -1208,12 +1316,17 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
           <t>601012_隆基绿能_2022年年度报告（修订版）.pdf @9; 603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -1247,12 +1360,18 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
+          <t>归属于本行普通股股东的每股净资产（元/股） = 21.89
+资产总额 = 5,769,270百万元</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
           <t>000001_平安银行_2024年年度报告.pdf @16</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr"/>
       <c r="I20" s="6" t="inlineStr"/>
       <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -1288,12 +1407,17 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净资产 = 244,637,811,032.18元</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2025年年度报告.pdf @6; 601012_隆基绿能_2025年年度报告.pdf @13</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -1329,12 +1453,20 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 25.28%
+归属于上市公司股东的净利润（元） = 26,690,661,397.42
+经营活动产生的现金流量净额（元） = 24,431,136,261.48
+总资产（元） = 152,714,727,880.22</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
           <t>000858_五 粮 液_2022年年度报告.pdf @7; 002594_比亚迪_2022年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr"/>
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -1368,12 +1500,21 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 19,762,103,017.38元
+营业利润 = 52,006,935,659.54元
+利润总额 = 52,386,185,416.63元
+归属于上市公司股 东的净资产 = 242,691,342,204.55元
+归属于上市公司股 东的每股净资产 = 21.00</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
           <t>000002_万科A_2022年年度报告.pdf @12</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr"/>
       <c r="I23" s="6" t="inlineStr"/>
       <c r="J23" s="6" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -1409,12 +1550,22 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
+          <t>投资活动产生的现金流量净额 = -13,326,365,843.11元
+筹资活动产生的现金流量净额 = 8,156,248,181.45元
+经营活动现金流入小计 = 243,587,978,384.02元
+经营活动现金流出小计 = 230,860,368,064.68元
+投资活动现金流入小计 = 10,037,921,670.41元
+投资活动现金流出小计 = 23,364,287,513.52元</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
           <t>002475_立讯精密_2022年年度报告.pdf @26; 002475_立讯精密_2024年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
       <c r="I24" s="6" t="inlineStr"/>
       <c r="J24" s="6" t="inlineStr"/>
+      <c r="K24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
@@ -1448,12 +1599,20 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每 股收益（元／股） = 2.82
+稀释每股收益（元／股） = 2.82
+加权平均净资产收益率（%） = 20.62
+扣除非经常性损益后的加权平 均净资产收益率（%） = 19.32</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
       <c r="I25" s="6" t="inlineStr"/>
       <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -1489,12 +1648,20 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每股收益（元／股） = 1.75
+稀释每股收益（元／股） = 1.83
+加权平均净资产收益率（%） = 20.87
+扣除非经常性损益后的加权平均净资产收益率（%） = 19.97</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
           <t>600887_伊利股份_内蒙古伊利实业集团股份有限公司2024年年度报告.pdf @7; 600887_伊利股份_内蒙古伊利实业集团股份有限公司2025年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr"/>
       <c r="I26" s="6" t="inlineStr"/>
       <c r="J26" s="6" t="inlineStr"/>
+      <c r="K26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -1528,12 +1695,17 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
           <t>601088_中国神华_中国神华2023年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr"/>
       <c r="I27" s="6" t="inlineStr"/>
       <c r="J27" s="6" t="inlineStr"/>
+      <c r="K27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -1567,12 +1739,17 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净资产（千元） = 162,878,825</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
           <t>000333_美的集团_2023年年度报告.pdf @10</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr"/>
       <c r="I28" s="6" t="inlineStr"/>
       <c r="J28" s="6" t="inlineStr"/>
+      <c r="K28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -1606,12 +1783,20 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净利润 = 82,320,067,101.68元
+归属于上市公司股东的扣除非 经常性损益的净利润 = 82,293,107,655.25元
+经营活动产生的现金流量净额 = 61,522,204,989.35元
+总资产 = 303,834,844,021.44元</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2025年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr"/>
       <c r="I29" s="6" t="inlineStr"/>
       <c r="J29" s="6" t="inlineStr"/>
+      <c r="K29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -1645,12 +1830,17 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
           <t>600276_恒瑞医药_恒瑞医药2024年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr"/>
       <c r="I30" s="6" t="inlineStr"/>
       <c r="J30" s="6" t="inlineStr"/>
+      <c r="K30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
@@ -1684,12 +1874,17 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 62,791,872,697.72元</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
       <c r="I31" s="6" t="inlineStr"/>
       <c r="J31" s="6" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -1725,12 +1920,17 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
           <t>601088_中国神华_中国神华2022年度报告.pdf @7; 601088_中国神华_中国神华2023年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr"/>
       <c r="I32" s="6" t="inlineStr"/>
       <c r="J32" s="6" t="inlineStr"/>
+      <c r="K32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -1764,12 +1964,18 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
+          <t>稀释每股收益（元/股） = 4.92
+加权平均净资产收益率 = 22.23%</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
           <t>000333_美的集团_2023年年度报告.pdf @10</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr"/>
       <c r="I33" s="6" t="inlineStr"/>
       <c r="J33" s="6" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -1805,12 +2011,22 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的净利润 = 32,496,172,808.65元
+归属于上市公司股 东的扣除非经常性 损益的净利润 = 32,507,551,977.06元
+经营活动产生的现 金流量净额 = 59,648,468,284.22元
+总资产 = 566,071,979,792.34元
+归属于上市公司 股东的净利润 = 27,238,970,860.70元
+归属于上市公司 股东的扣除非经 常性损益的净利 润 = 27,508,231,223.76元</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
           <t>600900_长江电力_长江电力2023年年度报告.pdf @6; 600900_长江电力_长江电力2024年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr"/>
       <c r="I34" s="6" t="inlineStr"/>
       <c r="J34" s="6" t="inlineStr"/>
+      <c r="K34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -1844,12 +2060,17 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净 资产 = 46,589,953,393.31元</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr"/>
       <c r="I35" s="6" t="inlineStr"/>
       <c r="J35" s="6" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -1883,12 +2104,18 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
+          <t>归属于本行普通股股东的每股净资产（元/股） = 23.25
+资产总额 = 5,925,777百万元</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
           <t>000001_平安银行_2025年年度报告.pdf @17</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr"/>
       <c r="I36" s="6" t="inlineStr"/>
       <c r="J36" s="6" t="inlineStr"/>
+      <c r="K36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -1924,12 +2151,17 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净资产（元） = 111,029,299,000.00</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
           <t>002594_比亚迪_2022年年度报告.pdf @8; 300760_迈瑞医疗_2023年年度报告.pdf @19</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr"/>
       <c r="I37" s="6" t="inlineStr"/>
       <c r="J37" s="6" t="inlineStr"/>
+      <c r="K37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -1963,12 +2195,17 @@
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 32,507,551,977.06元</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
           <t>600900_长江电力_长江电力2024年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr"/>
       <c r="I38" s="6" t="inlineStr"/>
       <c r="J38" s="6" t="inlineStr"/>
+      <c r="K38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -2002,12 +2239,18 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
+          <t>稀释每股收益（元/股） = 1.370
+加权平均净资产收益率 = 19.62%</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
           <t>002415_海康威视_2022年年度报告.pdf @10</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr"/>
       <c r="I39" s="6" t="inlineStr"/>
       <c r="J39" s="6" t="inlineStr"/>
+      <c r="K39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
@@ -2043,12 +2286,20 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每 股收益（元／股） = 0.5183
+稀释每股收益（元／股） = 0.7058
+加权平均净资产收益率（%） = 6.85
+扣除非经常性损益后的加权平 均净资产收益率（%） = 6.64</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
           <t>600031_三一重工_三一重工股份有限公司2023年年度报告.pdf @5; 600031_三一重工_三一重工股份有限公司2024年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr"/>
       <c r="I40" s="6" t="inlineStr"/>
       <c r="J40" s="6" t="inlineStr"/>
+      <c r="K40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -2082,12 +2333,20 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净利润 = 9,431,064,679.78元
+归属于上市公司股东的扣除非经 常性损益的净利润 = 8,585,692,731.44元
+经营活动产生的现金流量净额 = 13,420,320,580.36元
+总资产 = 130,965,302,299.22元</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
           <t>600887_伊利股份_内蒙古伊利实业集团股份有限公司2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr"/>
       <c r="I41" s="6" t="inlineStr"/>
       <c r="J41" s="6" t="inlineStr"/>
+      <c r="K41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -2123,12 +2382,17 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净资产（元） = 114,025,058,788.17</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
           <t>000858_五 粮 液_2022年年度报告.pdf @7; 002594_比亚迪_2022年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr"/>
       <c r="I42" s="6" t="inlineStr"/>
       <c r="J42" s="6" t="inlineStr"/>
+      <c r="K42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
@@ -2164,12 +2428,22 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 16.14%
+归属于上市公司股东的净利润（元） = 16,622,448,000.00
+经营活动产生的现金流量净额（元） = 140,837,657,000.00
+总资产（元） = 493,860,646,000.00
+归属于上市公司股东的净 利润 = 8,813,713,033.51元
+归属于上市公司股东的扣 除非经常性损益的净利润 = 8,260,289,685.19元</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
           <t>002594_比亚迪_2022年年度报告.pdf @8; 603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr"/>
       <c r="I43" s="6" t="inlineStr"/>
       <c r="J43" s="6" t="inlineStr"/>
+      <c r="K43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -2205,12 +2479,17 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
           <t>000858_五 粮 液_2022年年度报告.pdf @7; 002594_比亚迪_2022年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr"/>
       <c r="I44" s="6" t="inlineStr"/>
       <c r="J44" s="6" t="inlineStr"/>
+      <c r="K44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -2246,12 +2525,22 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的每股净 资产 = 17.09
+归属于上市公司股 东的每股净资产 = 21.00
+全面摊薄净资产收 益率 = 9.32%
+加权平均净资产收 益率 = 9.48%
+资产总额 = 1,286,259,859,765.82
+资产负债率 = 73.66%</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
           <t>000002_万科A_2022年年度报告.pdf @12; 000002_万科A_2024年年度报告.pdf @11</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr"/>
       <c r="I45" s="6" t="inlineStr"/>
       <c r="J45" s="6" t="inlineStr"/>
+      <c r="K45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -2285,12 +2574,18 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的扣 除非经常性损益的净利润 = 8,260,289,685.19元
+归属于上市公司股东的净 资产 = 46,589,953,393.31元</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr"/>
       <c r="I46" s="6" t="inlineStr"/>
       <c r="J46" s="6" t="inlineStr"/>
+      <c r="K46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -2324,12 +2619,17 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
           <t>002475_立讯精密_2024年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H47" s="6" t="inlineStr"/>
       <c r="I47" s="6" t="inlineStr"/>
       <c r="J47" s="6" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
@@ -2363,12 +2663,17 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净资产 = 54,655,690,475.89元</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
           <t>600887_伊利股份_内蒙古伊利实业集团股份有限公司2025年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H48" s="6" t="inlineStr"/>
       <c r="I48" s="6" t="inlineStr"/>
       <c r="J48" s="6" t="inlineStr"/>
+      <c r="K48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -2402,12 +2707,20 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的加权平均净资产收益率（%） = 19.36
+基本每股收益（元／股） = 1.64
+稀释每股收益（元／股） = 1.64
+扣除非经常性损益后的基本每股收益（元／股） = 1.57</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
           <t>600887_伊利股份_内蒙古伊利实业集团股份有限公司2023年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr"/>
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="6" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -2443,12 +2756,17 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
           <t>000858_五 粮 液_2022年年度报告.pdf @7; 601012_隆基绿能_2023年年度报告.pdf @11</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr"/>
       <c r="I50" s="6" t="inlineStr"/>
       <c r="J50" s="6" t="inlineStr"/>
+      <c r="K50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -2484,12 +2802,22 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每股收益 （元／股） = 1.3669
+扣除非经常性损益后的基本每 股收益（元／股） = 1.3286
+稀释每股收益（元／股） = 1.4101
+加权平均净资产收益率（%） = 15.90
+扣除非经常性损益后的加权平均净资 产收益率（%） = 15.41
+扣除非经常性损益后的加权平 均净资产收益率（%） = 15.72</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
           <t>600900_长江电力_长江电力2024年年度报告.pdf @6; 600900_长江电力_长江电力2025年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr"/>
       <c r="I51" s="6" t="inlineStr"/>
       <c r="J51" s="6" t="inlineStr"/>
+      <c r="K51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
@@ -2525,12 +2853,22 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
+          <t>归属于本行普通股股东的每股净资产（元/股） = 18.80
+资产总额 = 5,321,514百万元
+归属于上市公司股 东的净利润 = 62,716,443,738.27元
+归属于上市公司股 东的扣除非经常性 损益的净利润 = 62,791,872,697.72元
+经营活动产生的现 金流量净额 = 36,698,595,830.03元
+总资产 = 254,364,804,995.25元</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
           <t>000001_平安银行_2022年年度报告.pdf @18; 600519_贵州茅台_贵州茅台2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr"/>
       <c r="I52" s="6" t="inlineStr"/>
       <c r="J52" s="6" t="inlineStr"/>
+      <c r="K52" s="6" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -2564,12 +2902,20 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的加权平 均净资产收益率（%） = 34.20
+基本每股收益（元／股） = 59.49
+稀释每股收益（元／股） = 59.49
+扣除非经常性损益后的基本每 股收益（元／股） = 59.51</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2023年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr"/>
       <c r="I53" s="6" t="inlineStr"/>
       <c r="J53" s="6" t="inlineStr"/>
+      <c r="K53" s="6" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -2603,12 +2949,17 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
+          <t>归属于本行普通股股东的每股净资产（元/股） = 18.80</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
           <t>000001_平安银行_2022年年度报告.pdf @18</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr"/>
       <c r="I54" s="6" t="inlineStr"/>
       <c r="J54" s="6" t="inlineStr"/>
+      <c r="K54" s="6" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
@@ -2642,12 +2993,17 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
           <t>002594_比亚迪_2022年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr"/>
       <c r="I55" s="6" t="inlineStr"/>
       <c r="J55" s="6" t="inlineStr"/>
+      <c r="K55" s="6" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
@@ -2681,12 +3037,18 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
+          <t>稀释每股收益（元/股） = 11.58
+加权平均净资产收益率 = 24.13%</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
           <t>300750_宁德时代_2024年年度报告.pdf @9</t>
         </is>
       </c>
-      <c r="H56" s="6" t="inlineStr"/>
       <c r="I56" s="6" t="inlineStr"/>
       <c r="J56" s="6" t="inlineStr"/>
+      <c r="K56" s="6" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n">
@@ -2720,12 +3082,17 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
           <t>600031_三一重工_三一重工股份有限公司2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr"/>
       <c r="I57" s="6" t="inlineStr"/>
       <c r="J57" s="6" t="inlineStr"/>
+      <c r="K57" s="6" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n">
@@ -2759,12 +3126,18 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 62,791,872,697.72元
+归属于上市公司股 东的净资产 = 197,506,672,396.00元</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr"/>
       <c r="I58" s="6" t="inlineStr"/>
       <c r="J58" s="6" t="inlineStr"/>
+      <c r="K58" s="6" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
@@ -2800,12 +3173,22 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 22.23%
+归属于上市公司股东的净利润（千元） = 33,719,935
+经营活动产生的现金流量净额（千元） = 57,902,611
+总资产（千元） = 486,038,184
+归属于上市公司股东的净利润（元） = 13,365,651,026.16
+经营活动产生的现金流量净额（元） = 27,116,908,208.53</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
           <t>000333_美的集团_2023年年度报告.pdf @10; 002475_立讯精密_2024年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr"/>
       <c r="I59" s="6" t="inlineStr"/>
       <c r="J59" s="6" t="inlineStr"/>
+      <c r="K59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -2841,12 +3224,18 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的扣除非 经常性损益的净利润 = 11,068,321,695.12元
+归属于上市公司 股东的扣除非经 常性损益的净利 润 = 13,240,556,954.42元</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
           <t>600887_伊利股份_内蒙古伊利实业集团股份有限公司2025年年度报告.pdf @7; 603259_药明康德_2025年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H60" s="6" t="inlineStr"/>
       <c r="I60" s="6" t="inlineStr"/>
       <c r="J60" s="6" t="inlineStr"/>
+      <c r="K60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -2880,12 +3269,18 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 22.23%
+归属于上市公司股东的净资产（千元） = 162,878,825</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
           <t>000333_美的集团_2023年年度报告.pdf @10</t>
         </is>
       </c>
-      <c r="H61" s="6" t="inlineStr"/>
       <c r="I61" s="6" t="inlineStr"/>
       <c r="J61" s="6" t="inlineStr"/>
+      <c r="K61" s="6" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -2919,12 +3314,18 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 22.23%
+归属于上市公司股东的净资产（千元） = 162,878,825</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
           <t>000333_美的集团_2023年年度报告.pdf @10</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr"/>
       <c r="I62" s="6" t="inlineStr"/>
       <c r="J62" s="6" t="inlineStr"/>
+      <c r="K62" s="6" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -2960,12 +3361,17 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净资产（元） = 69,327,010,925.99</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
           <t>002475_立讯精密_2024年年度报告.pdf @8; 002594_比亚迪_2022年年度报告.pdf @8</t>
         </is>
       </c>
-      <c r="H63" s="6" t="inlineStr"/>
       <c r="I63" s="6" t="inlineStr"/>
       <c r="J63" s="6" t="inlineStr"/>
+      <c r="K63" s="6" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -2999,12 +3405,17 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的净资产 = 64,965,662千元</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
           <t>600031_三一重工_三一重工股份有限公司2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H64" s="6" t="inlineStr"/>
       <c r="I64" s="6" t="inlineStr"/>
       <c r="J64" s="6" t="inlineStr"/>
+      <c r="K64" s="6" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
@@ -3040,12 +3451,18 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的扣除非经常 性损益的净利润 = 3,126,760千元
+归属于上市公司股东的扣 除非经常性损益的净利润 = 8,260,289,685.19元</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
           <t>600031_三一重工_三一重工股份有限公司2022年年度报告.pdf @5; 603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H65" s="6" t="inlineStr"/>
       <c r="I65" s="6" t="inlineStr"/>
       <c r="J65" s="6" t="inlineStr"/>
+      <c r="K65" s="6" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
@@ -3079,12 +3496,17 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
           <t>300760_迈瑞医疗_2024年年度报告.pdf @21</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr"/>
       <c r="I66" s="6" t="inlineStr"/>
       <c r="J66" s="6" t="inlineStr"/>
+      <c r="K66" s="6" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n">
@@ -3120,12 +3542,20 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每股 收益（元／股） = -1.16
+稀释每股收益（元／股） = -1.14
+加权平均净资产收益率（%） = -13.10
+扣除非经常性损益后的加权平均 净资产收益率（%） = -13.30</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
           <t>601012_隆基绿能_2023年年度报告.pdf @12; 601012_隆基绿能_2024年年度报告（修订版）.pdf @11</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr"/>
       <c r="I67" s="6" t="inlineStr"/>
       <c r="J67" s="6" t="inlineStr"/>
+      <c r="K67" s="6" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n">
@@ -3161,12 +3591,19 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后归属于上 市公司股东的净利润 = (45,393,719,289.83)元
+营业利润 = (45,643,796,280.61)元
+利润总额 = (47,186,559,181.39)元</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
           <t>000002_万科A_2024年年度报告.pdf @11; 300760_迈瑞医疗_2024年年度报告.pdf @21</t>
         </is>
       </c>
-      <c r="H68" s="6" t="inlineStr"/>
       <c r="I68" s="6" t="inlineStr"/>
       <c r="J68" s="6" t="inlineStr"/>
+      <c r="K68" s="6" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n">
@@ -3202,12 +3639,20 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每 股收益（元／股） = 0.9616
+稀释每股收益（元／股） = 0.9834
+加权平均净资产收益率（%） = 11.18
+扣除非经常性损益后的加权平 均净资产收益率（%） = 10.93</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
           <t>600031_三一重工_三一重工股份有限公司2024年年度报告.pdf @5; 600031_三一重工_三一重工股份有限公司2025年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H69" s="6" t="inlineStr"/>
       <c r="I69" s="6" t="inlineStr"/>
       <c r="J69" s="6" t="inlineStr"/>
+      <c r="K69" s="6" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n">
@@ -3241,12 +3686,17 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的扣除非经常 性损益的净利润 = 3,126,760千元</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
           <t>600031_三一重工_三一重工股份有限公司2022年年度报告.pdf @5</t>
         </is>
       </c>
-      <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="6" t="inlineStr"/>
       <c r="J70" s="6" t="inlineStr"/>
+      <c r="K70" s="6" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n">
@@ -3280,12 +3730,18 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
+          <t>稀释每股收益（元/股） = 6.876
+加权平均净资产收益率 = 25.28%</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
           <t>000858_五 粮 液_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="6" t="inlineStr"/>
       <c r="J71" s="6" t="inlineStr"/>
+      <c r="K71" s="6" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -3321,12 +3777,19 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司 股东的扣除非经 常性损益的净利 润 = 27,508,231,223.76元
+归属于上市公司股东的净资产（千元） = 246,930,033
+归属于上市公司 股东的净资产 = 201,330,025,517.69元</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
           <t>300750_宁德时代_2024年年度报告.pdf @9; 600900_长江电力_长江电力2023年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="6" t="inlineStr"/>
       <c r="J72" s="6" t="inlineStr"/>
+      <c r="K72" s="6" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n">
@@ -3360,12 +3823,18 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 22.23%
+归属于上市公司股东的净资产（千元） = 162,878,825</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
           <t>000333_美的集团_2023年年度报告.pdf @10</t>
         </is>
       </c>
-      <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="6" t="inlineStr"/>
+      <c r="K73" s="6" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n">
@@ -3401,12 +3870,20 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的扣除非 经常性损益的净利润 = 82,293,107,655.25元
+归属于上市公司股东的扣除非经常性 损益的净利润 = -7,361,963,984.28元
+利润总额 = 114,755,261,605.08元
+归属于上市公司股东的净资产 = 244,637,811,032.18元</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2025年年度报告.pdf @6; 601012_隆基绿能_2025年年度报告.pdf @13</t>
         </is>
       </c>
-      <c r="H74" s="6" t="inlineStr"/>
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr"/>
+      <c r="K74" s="6" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n">
@@ -3440,12 +3917,19 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的每股净 资产 = 17.09
+资产总额 = 1,286,259,859,765.82
+资产负债率 = 73.66%</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
           <t>000002_万科A_2024年年度报告.pdf @11</t>
         </is>
       </c>
-      <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="6" t="inlineStr"/>
       <c r="J75" s="6" t="inlineStr"/>
+      <c r="K75" s="6" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n">
@@ -3479,12 +3963,17 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
+          <t>扣除与主营业务无关的业 务收入和不具备商业实质 的收入后的营业收入 = 81,211,823,906.59元</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
           <t>601012_隆基绿能_2024年年度报告（修订版）.pdf @11</t>
         </is>
       </c>
-      <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="6" t="inlineStr"/>
       <c r="J76" s="6" t="inlineStr"/>
+      <c r="K76" s="6" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n">
@@ -3518,12 +4007,20 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每股收益 （元／股） = 1.3669
+稀释每股收益（元／股） = 1.4101
+加权平均净资产收益率（%） = 15.90
+扣除非经常性损益后的加权平均净资 产收益率（%） = 15.41</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
           <t>600900_长江电力_长江电力2025年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H77" s="6" t="inlineStr"/>
       <c r="I77" s="6" t="inlineStr"/>
       <c r="J77" s="6" t="inlineStr"/>
+      <c r="K77" s="6" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
@@ -3557,12 +4054,20 @@
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的加权平均 净资产收益率（%） = 13.71
+基本每股收益（元／股） = 1.19
+稀释每股收益（元／股） = 1.18
+扣除非经常性损益后的基本每股 收益（元／股） = 1.14</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
           <t>600276_恒瑞医药_恒瑞医药2025年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H78" s="6" t="inlineStr"/>
       <c r="I78" s="6" t="inlineStr"/>
       <c r="J78" s="6" t="inlineStr"/>
+      <c r="K78" s="6" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n">
@@ -3596,12 +4101,17 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
+          <t>（同表无口径相近的其他行）</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H79" s="6" t="inlineStr"/>
       <c r="I79" s="6" t="inlineStr"/>
       <c r="J79" s="6" t="inlineStr"/>
+      <c r="K79" s="6" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n">
@@ -3635,12 +4145,18 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股东的扣除非经 常性损益的净利润 = 8,585,692,731.44元
+归属于上市公司股东的净资产 = 50,267,883,832.15元</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
           <t>600887_伊利股份_内蒙古伊利实业集团股份有限公司2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H80" s="6" t="inlineStr"/>
       <c r="I80" s="6" t="inlineStr"/>
       <c r="J80" s="6" t="inlineStr"/>
+      <c r="K80" s="6" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n">
@@ -3674,12 +4190,17 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
+          <t>营业成本 = 百万元</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
           <t>601088_中国神华_中国神华2022年度报告.pdf @29</t>
         </is>
       </c>
-      <c r="H81" s="6" t="inlineStr"/>
       <c r="I81" s="6" t="inlineStr"/>
       <c r="J81" s="6" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
@@ -3713,12 +4234,18 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
+          <t>归属于上市公司股 东的扣除非经常性 损益的净利润 = 21,392,344,535.58元
+归属于上市公司股 东的净资产 = 185,488,250,616.82元</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
           <t>600900_长江电力_长江电力2022年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H82" s="6" t="inlineStr"/>
       <c r="I82" s="6" t="inlineStr"/>
       <c r="J82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n">
@@ -3754,12 +4281,20 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
+          <t>加权平均净资产收益率 = 25.28%
+归属于上市公司股东的净利润（元） = 26,690,661,397.42
+经营活动产生的现金流量净额（元） = 24,431,136,261.48
+总资产（元） = 152,714,727,880.22</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
           <t>000858_五 粮 液_2022年年度报告.pdf @7; 002415_海康威视_2022年年度报告.pdf @10</t>
         </is>
       </c>
-      <c r="H83" s="6" t="inlineStr"/>
       <c r="I83" s="6" t="inlineStr"/>
       <c r="J83" s="6" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
@@ -3793,20 +4328,28 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的基本每 股收益（元／股） = 0.9407
+稀释每股收益（元／股） = 0.9370
+加权平均净资产收益率（%） = 11.73
+扣除非经常性损益后的加权平 均净资产收益率（%） = 11.77</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
           <t>600900_长江电力_长江电力2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H84" s="6" t="inlineStr"/>
       <c r="I84" s="6" t="inlineStr"/>
       <c r="J84" s="6" t="inlineStr"/>
+      <c r="K84" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:I84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I5:J84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓,✗,存疑"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3820,19 +4363,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3848,7 +4392,8 @@
           <t>这几条首轮标为「存疑」，指出的缺陷（比率型指标误标货币单位）其后已在数据集中修复。旧标注对应的是修复前的数据，若直接拿来配对，会把版本差异算成标注者分歧。请按当前内容重新判定。填写说明：只需填黄色三列，用下拉选择 ✓ / ✗ / 存疑，有疑问时在备注列写一句原因。第4行为示例行（不计入统计）。请独立判定——不要参考另一位标注者的结果，也不要互相商量，否则一致性系数失去意义。
 【答案正确?】标准答案与原文是否相符（数值、行标签、年份、量纲）。相符✓，不符✗。
 【唯一合理答案?】在问题的字面表述下，标准答案是否是唯一站得住的答案。是✓；若一个称职的分析师可能给出另一个同样站得住的答案，判✗并在备注写出那个答案。常见歧义来源：①指标口径（归母净资产／所有者权益合计、营业收入／营业总收入）；②合并报表与母公司报表；③上年数是追溯调整后还是原披露数；④同一年数字在本年报与次年年报的上年同期栏都出现，取哪一处。
-注意这两列相互独立：答案可以完全正确，但问题本身有歧义（判 ✓ / ✗）。证据原文列是自动匹配的 gold 三元组；表名若读不出计量单位，请对照原PDF确认量纲。</t>
+注意这两列相互独立：答案可以完全正确，但问题本身有歧义。
+【同表相近行】列出了同一张表里口径相近的其他科目及其数值——判歧义时先看这一列，多数情况无需打开源PDF。仅当表名读不出计量单位、或需确认上年数是否追溯调整时，才需对照原PDF。</t>
         </is>
       </c>
     </row>
@@ -3885,20 +4430,25 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>同表相近行（判歧义用）</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>来源（文件@页）</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>答案正确?</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>唯一合理答案?</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -3937,22 +4487,28 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
+          <t>营业总收入 = 164,699百万元
+利息净收入 = 116,061百万元</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
           <t>000001_平安银行_2023年年度报告.pdf @15</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>数值与原文一致；「营业收入」在该表中口径唯一</t>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>数值与原文一致；该表虽有「营业总收入」，但本行两者同值，不构成歧义</t>
         </is>
       </c>
     </row>
@@ -3988,12 +4544,19 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
+          <t>【三一重工 三一重工股份有限公司2024年年度报告】加权平均净资产收益率（%） = 8.54
+【三一重工 三一重工股份有限公司2024年年度报告】扣除非经常性损益后的加权平 均净资产收益率（%） = 7.62
+【三一重工 三一重工股份有限公司2024年年度报告】扣除非经常性损益后的基本每 股收益（元／股） = 0.6297</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
           <t>600031_三一重工_三一重工股份有限公司2024年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -4027,12 +4590,20 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的加权平 均净资产收益率（%） = 19.32
+基本每股收益（元／股） = 3.01
+稀释每股收益（元／股） = 2.82
+扣除非经常性损益后的基本每 股收益（元／股） = 2.82</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
           <t>603259_药明康德_2022年年度报告.pdf @7</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -4066,12 +4637,20 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的加权平均 净资产收益率（%） = 16.33
+基本每股收益（元／股） = 1.42
+稀释每股收益（元／股） = 1.42
+扣除非经常性损益后的基本每股 收益（元／股） = 1.43</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
           <t>601012_隆基绿能_2023年年度报告.pdf @12</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -4105,20 +4684,28 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
+          <t>扣除非经常性损益后的加权平均 净资产收益率（%） = 32.52
+基本每股收益（元／股） = 65.66
+稀释每股收益（元／股） = 65.66
+扣除非经常性损益后的基本每股 收益（元／股） = 65.64</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
           <t>600519_贵州茅台_贵州茅台2025年年度报告.pdf @6</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:I8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I5:J8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓,✗,存疑"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>